<commit_message>
Corrected legal status field name in metadata
</commit_message>
<xml_diff>
--- a/reference files/baseline_extract_meta.xlsx
+++ b/reference files/baseline_extract_meta.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andrew.Hood\OneDrive - Midlands and Lancashire CSU\Working Projects\MH inpat modelling\main repo\nhse_mh_inpat_model\reference files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/alexander_lawless1_nhs_net/Documents/Work/1. Projects/2024_25/mental_health_shiny_app/nhse_mh_inpat_model/reference files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ED731DF-BF7E-461D-ACEC-68BFD76A1DE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{9ED731DF-BF7E-461D-ACEC-68BFD76A1DE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{04B45AE9-7867-4D6F-A459-EC496C4A1AA0}"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="10940" xr2:uid="{01FA3479-5CA2-470F-B017-4BB0F2949246}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{01FA3479-5CA2-470F-B017-4BB0F2949246}"/>
   </bookViews>
   <sheets>
     <sheet name="baseline_extract_meta" sheetId="1" r:id="rId1"/>
@@ -97,9 +97,6 @@
     <t>NHS determined by codes starting with 'R'. All others independent</t>
   </si>
   <si>
-    <t>legal_status_code</t>
-  </si>
-  <si>
     <t>Whether patient is formally detained under MHA or not</t>
   </si>
   <si>
@@ -167,6 +164,9 @@
   </si>
   <si>
     <t>Raw extract constrained to any midlands resident OR admission to midlands based provider. Last known LSOA used when missing from record.</t>
+  </si>
+  <si>
+    <t>legal_status_group</t>
   </si>
 </sst>
 </file>
@@ -1028,15 +1028,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D586B6A4-BFFC-439D-84AB-BFCC871E2CAE}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.81640625" customWidth="1"/>
-    <col min="2" max="2" width="75.90625" customWidth="1"/>
-    <col min="3" max="3" width="52.08984375" customWidth="1"/>
-    <col min="4" max="4" width="26.81640625" customWidth="1"/>
+    <col min="1" max="1" width="26.77734375" customWidth="1"/>
+    <col min="2" max="2" width="75.88671875" customWidth="1"/>
+    <col min="3" max="3" width="52.109375" customWidth="1"/>
+    <col min="4" max="4" width="26.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1050,7 +1050,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1058,10 +1058,10 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -1069,10 +1069,10 @@
         <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1083,7 +1083,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -1094,7 +1094,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -1105,7 +1105,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>17</v>
       </c>
@@ -1119,7 +1119,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1133,92 +1133,98 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" t="s">
         <v>25</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>26</v>
       </c>
-      <c r="C9" t="s">
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
+      <c r="B10" t="s">
         <v>28</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>29</v>
       </c>
-      <c r="C10" t="s">
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
+      <c r="B11" t="s">
         <v>31</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>32</v>
       </c>
-      <c r="C11" t="s">
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
+      <c r="B12" t="s">
         <v>34</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>35</v>
       </c>
-      <c r="C12" t="s">
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
+      <c r="B13" t="s">
         <v>37</v>
       </c>
-      <c r="B13" t="s">
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
+      <c r="B14" t="s">
         <v>39</v>
       </c>
-      <c r="B14" t="s">
+      <c r="D14" t="s">
         <v>40</v>
       </c>
-      <c r="D14" t="s">
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
+      <c r="B15" t="s">
         <v>42</v>
       </c>
-      <c r="B15" t="s">
+      <c r="D15" t="s">
         <v>43</v>
       </c>
-      <c r="D15" t="s">
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
+      <c r="B16" t="s">
         <v>45</v>
       </c>
-      <c r="B16" t="s">
+      <c r="D16" t="s">
         <v>46</v>
-      </c>
-      <c r="D16" t="s">
-        <v>47</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{37c354b2-85b0-47f5-b222-07b48d774ee3}" enabled="0" method="" siteId="{37c354b2-85b0-47f5-b222-07b48d774ee3}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Added ICB code and name format instructions
</commit_message>
<xml_diff>
--- a/reference files/baseline_extract_meta.xlsx
+++ b/reference files/baseline_extract_meta.xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/alexander_lawless1_nhs_net/Documents/Work/1. Projects/2024_25/mental_health_shiny_app/nhse_mh_inpat_model/reference files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{9ED731DF-BF7E-461D-ACEC-68BFD76A1DE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{04B45AE9-7867-4D6F-A459-EC496C4A1AA0}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{9ED731DF-BF7E-461D-ACEC-68BFD76A1DE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E636C79-A47E-4CA4-B577-8466206E7A1C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{01FA3479-5CA2-470F-B017-4BB0F2949246}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{01FA3479-5CA2-470F-B017-4BB0F2949246}"/>
   </bookViews>
   <sheets>
     <sheet name="baseline_extract_meta" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
   <si>
     <t>Field</t>
   </si>
@@ -163,10 +176,13 @@
     <t>Derived from MHS504 and MHS518 tables (MHSDS)</t>
   </si>
   <si>
-    <t>Raw extract constrained to any midlands resident OR admission to midlands based provider. Last known LSOA used when missing from record.</t>
-  </si>
-  <si>
     <t>legal_status_group</t>
+  </si>
+  <si>
+    <t>Raw extract constrained to any midlands resident OR admission to midlands based provider. Last known LSOA used when missing from record. Name must include 3-digit area code as a prefix e.g. "AT1: Anytown ICB_1".</t>
+  </si>
+  <si>
+    <t>Raw extract constrained to any midlands resident OR admission to midlands based provider. Last known LSOA used when missing from record. Must be a capitalised 3-digit ICB code, matching the following format: "ABC" or "AT1" - can include 3 letters or 2 letters and a number.</t>
   </si>
 </sst>
 </file>
@@ -1058,7 +1074,7 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -1069,7 +1085,7 @@
         <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -1135,7 +1151,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B9" t="s">
         <v>25</v>

</xml_diff>